<commit_message>
fixed innacurate proportion values
</commit_message>
<xml_diff>
--- a/data/sample_proportions.xlsx
+++ b/data/sample_proportions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arondiamond/Desktop/Fellowship/norovirus/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{294CE639-A135-2245-B2FE-91331E88B9EE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F45CD8FE-32A0-0C42-843B-F1E0037CF13A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="80" yWindow="500" windowWidth="21200" windowHeight="16400" xr2:uid="{5D9D4F30-FFDC-1F43-9897-27E196BDB714}"/>
   </bookViews>
@@ -2544,13 +2544,13 @@
         <v>0.3</v>
       </c>
       <c r="E51" s="1">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="F51" s="1">
         <v>0.1</v>
       </c>
       <c r="G51" s="1">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="H51" s="1">
         <v>0</v>

</xml_diff>